<commit_message>
Five units on top of existing tools (funnel, ads budget, store P&L, RICE, LTV/CAC); RICE table in person-months; no layout shift on deep links; a11y heading order and contrast
</commit_message>
<xml_diff>
--- a/v6/files/r-rice-table.xlsx
+++ b/v6/files/r-rice-table.xlsx
@@ -480,7 +480,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>3. Усилия в человеко-неделях: сколько недель работы одного человека займёт идея.</t>
+          <t>3. Трудозатраты в человеко-месяцах всех, кто участвует. Работу заметно меньше месяца ставьте 0,5.</t>
         </is>
       </c>
     </row>
@@ -555,7 +555,7 @@
       </c>
       <c r="E1" s="3" t="inlineStr">
         <is>
-          <t>Усилия, человеко-недели</t>
+          <t>Трудозатраты, человеко-месяцы</t>
         </is>
       </c>
       <c r="F1" s="3" t="inlineStr">
@@ -590,7 +590,7 @@
         <v>80</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2">
         <f>IF(OR(A2="",E2=0,E2=""),"",ROUND(B2*C2*(D2/100)/E2,0))</f>
@@ -622,7 +622,7 @@
         <v>100</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="F3">
         <f>IF(OR(A3="",E3=0,E3=""),"",ROUND(B3*C3*(D3/100)/E3,0))</f>
@@ -654,7 +654,7 @@
         <v>50</v>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4">
         <f>IF(OR(A4="",E4=0,E4=""),"",ROUND(B4*C4*(D4/100)/E4,0))</f>

</xml_diff>